<commit_message>
Add DBZ-only rostered table (203 agents) to the Week 28 Sep-4 Oct shift snapshot
</commit_message>
<xml_diff>
--- a/2026-09-28/Snapshot_Sep28_Oct4.xlsx
+++ b/2026-09-28/Snapshot_Sep28_Oct4.xlsx
@@ -55,7 +55,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -77,11 +77,55 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -96,6 +140,8 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -488,25 +534,25 @@
           <t>All Agents DBZ - 248 Agents</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="6" t="n"/>
+      <c r="C1" s="6" t="n"/>
+      <c r="D1" s="6" t="n"/>
+      <c r="E1" s="6" t="n"/>
+      <c r="F1" s="6" t="n"/>
+      <c r="G1" s="6" t="n"/>
+      <c r="H1" s="7" t="n"/>
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Mirkl Rostered - 15 Agents</t>
         </is>
       </c>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="2" t="n"/>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="2" t="n"/>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="2" t="n"/>
+      <c r="L1" s="6" t="n"/>
+      <c r="M1" s="6" t="n"/>
+      <c r="N1" s="6" t="n"/>
+      <c r="O1" s="6" t="n"/>
+      <c r="P1" s="6" t="n"/>
+      <c r="Q1" s="6" t="n"/>
+      <c r="R1" s="7" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -866,13 +912,13 @@
           <t>KM Rostered - 30 Agents</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1056,9 +1102,206 @@
         <v>11</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>DBZ Rostered - 203 Agents</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Shifts</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>07:00-15:30</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>08:00-16:30</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>11:30-20:00</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>13:30-22:00</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Rostered</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>156</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>159</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>159</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>167</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>167</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>93</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="K1:R1"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>